<commit_message>
Refactor PQG reward calculation and enhance combat feedback
- Updated the `calculate_pqg_from_xp` function to improve accuracy in PQG rewards based on XP earned.
- Adjusted XP scaling factors for better balance in player progression.
- Enhanced the `CombatSystem` to provide clearer feedback when awarding PQG upon monster defeat.
- Added new unit tests to ensure the reliability of PQG calculations and their integration with combat mechanics.
- Modified existing tests to align with the updated XP and PQG reward system.
</commit_message>
<xml_diff>
--- a/weapon_types.xlsx
+++ b/weapon_types.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\info\Documents\Projects\dungeon-console\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_F56CE08520D019DA16317F948C4E9A2163C31231" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEEED51A-02E2-4DBE-B986-4670C78F2230}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="32340" yWindow="2505" windowWidth="21600" windowHeight="11175" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,7 +19,20 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Weapons!$A$1:$G$41</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -652,7 +665,7 @@
         <v>10</v>
       </c>
       <c r="F2" s="2">
-        <v>2</v>
+        <v>30</v>
       </c>
       <c r="G2" s="2">
         <v>2.5</v>

</xml_diff>